<commit_message>
conducted tesla model3 analysis for dynamic response test
</commit_message>
<xml_diff>
--- a/src/tools/xil-data-analysis/2020-Tesla-Model3/output-file/analysis-data.xlsx
+++ b/src/tools/xil-data-analysis/2020-Tesla-Model3/output-file/analysis-data.xlsx
@@ -2,30 +2,42 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" tabRatio="600" firstSheet="2" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20-40mph" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0-20mph" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50-70mph" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0-20mph" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10-30mph" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20-40mph" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="30-50mph" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="40-60mph" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50-70mph" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -39,12 +51,42 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -57,14 +99,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -427,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,13 +505,13 @@
         <v>0.25</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5999999999999979</v>
+        <v>0.6000000000000085</v>
       </c>
       <c r="C2" t="n">
         <v>0.25</v>
       </c>
       <c r="D2" t="n">
-        <v>37.20000000000041</v>
+        <v>36.7999999999986</v>
       </c>
     </row>
     <row r="3">
@@ -477,7 +525,7 @@
         <v>-0.25</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6999999999999602</v>
+        <v>37.79999999999787</v>
       </c>
     </row>
     <row r="4">
@@ -491,7 +539,7 @@
         <v>0.5</v>
       </c>
       <c r="D4" t="n">
-        <v>20.39999999999884</v>
+        <v>17.09999999999903</v>
       </c>
     </row>
     <row r="5">
@@ -505,7 +553,7 @@
         <v>-0.5</v>
       </c>
       <c r="D5" t="n">
-        <v>3.899999999999778</v>
+        <v>22.29999999999873</v>
       </c>
     </row>
     <row r="6">
@@ -519,7 +567,7 @@
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>9.100000000002069</v>
+        <v>9.000000000002046</v>
       </c>
     </row>
     <row r="7">
@@ -533,7 +581,7 @@
         <v>-1</v>
       </c>
       <c r="D7" t="n">
-        <v>0.1000000000000227</v>
+        <v>8.700000000001978</v>
       </c>
     </row>
     <row r="8">
@@ -547,7 +595,7 @@
         <v>1.5</v>
       </c>
       <c r="D8" t="n">
-        <v>6.20000000000141</v>
+        <v>6.100000000001387</v>
       </c>
     </row>
     <row r="9">
@@ -561,7 +609,7 @@
         <v>-1.5</v>
       </c>
       <c r="D9" t="n">
-        <v>0.7000000000001592</v>
+        <v>7.30000000000166</v>
       </c>
     </row>
     <row r="10">
@@ -575,7 +623,7 @@
         <v>1.6</v>
       </c>
       <c r="D10" t="n">
-        <v>6.100000000001387</v>
+        <v>5.700000000001296</v>
       </c>
     </row>
     <row r="11">
@@ -589,7 +637,7 @@
         <v>-1.6</v>
       </c>
       <c r="D11" t="n">
-        <v>0.9000000000002046</v>
+        <v>7.200000000001637</v>
       </c>
     </row>
     <row r="12">
@@ -617,7 +665,7 @@
         <v>-1.75</v>
       </c>
       <c r="D13" t="n">
-        <v>0.5000000000001137</v>
+        <v>5.800000000001319</v>
       </c>
     </row>
     <row r="14">
@@ -645,7 +693,7 @@
         <v>-2</v>
       </c>
       <c r="D15" t="n">
-        <v>0.6000000000001364</v>
+        <v>5.700000000001296</v>
       </c>
     </row>
     <row r="16">
@@ -659,7 +707,21 @@
         <v>2.25</v>
       </c>
       <c r="D16" t="n">
-        <v>5.400000000001228</v>
+        <v>4.700000000001069</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>-1</v>
+      </c>
+      <c r="B17" t="n">
+        <v>8.800000000002001</v>
+      </c>
+      <c r="C17" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>10.60000000000241</v>
       </c>
     </row>
   </sheetData>
@@ -673,7 +735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -700,16 +762,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.5999999999999979</v>
+        <v>0.3000000000000043</v>
       </c>
       <c r="C2" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>36.8000000000004</v>
+        <v>95.19999999999473</v>
       </c>
     </row>
     <row r="3">
@@ -723,7 +785,7 @@
         <v>-0.25</v>
       </c>
       <c r="D3" t="n">
-        <v>37.79999999999785</v>
+        <v>136.0000000000088</v>
       </c>
     </row>
     <row r="4">
@@ -734,10 +796,10 @@
         <v>0.3999999999999773</v>
       </c>
       <c r="C4" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>17.09999999999903</v>
+        <v>9.100000000002069</v>
       </c>
     </row>
     <row r="5">
@@ -745,13 +807,13 @@
         <v>-0.5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.2999999999999829</v>
+        <v>0.3000000000000682</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.5</v>
+        <v>-1</v>
       </c>
       <c r="D5" t="n">
-        <v>22.29999999999873</v>
+        <v>8.800000000002001</v>
       </c>
     </row>
     <row r="6">
@@ -759,13 +821,13 @@
         <v>1</v>
       </c>
       <c r="B6" t="n">
-        <v>0.1000000000000227</v>
+        <v>0.3000000000000682</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="D6" t="n">
-        <v>9.000000000002046</v>
+        <v>78.70000000001789</v>
       </c>
     </row>
     <row r="7">
@@ -773,13 +835,13 @@
         <v>-1</v>
       </c>
       <c r="B7" t="n">
-        <v>0.3000000000000682</v>
+        <v>0.2000000000000455</v>
       </c>
       <c r="C7" t="n">
-        <v>-1</v>
+        <v>-1.5</v>
       </c>
       <c r="D7" t="n">
-        <v>8.700000000001978</v>
+        <v>10.30000000000234</v>
       </c>
     </row>
     <row r="8">
@@ -787,13 +849,13 @@
         <v>1.5</v>
       </c>
       <c r="B8" t="n">
-        <v>0.1000000000000227</v>
+        <v>0.4000000000000909</v>
       </c>
       <c r="C8" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="D8" t="n">
-        <v>6.100000000001387</v>
+        <v>5.700000000001296</v>
       </c>
     </row>
     <row r="9">
@@ -804,10 +866,10 @@
         <v>0.2000000000000455</v>
       </c>
       <c r="C9" t="n">
-        <v>-1.5</v>
+        <v>-1.6</v>
       </c>
       <c r="D9" t="n">
-        <v>7.30000000000166</v>
+        <v>6.100000000001387</v>
       </c>
     </row>
     <row r="10">
@@ -815,13 +877,13 @@
         <v>1.6</v>
       </c>
       <c r="B10" t="n">
-        <v>0.2000000000000455</v>
+        <v>0.3000000000000682</v>
       </c>
       <c r="C10" t="n">
-        <v>1.6</v>
+        <v>1.75</v>
       </c>
       <c r="D10" t="n">
-        <v>5.700000000001296</v>
+        <v>5.300000000001205</v>
       </c>
     </row>
     <row r="11">
@@ -832,10 +894,10 @@
         <v>0.2000000000000455</v>
       </c>
       <c r="C11" t="n">
-        <v>-1.6</v>
+        <v>-1.75</v>
       </c>
       <c r="D11" t="n">
-        <v>7.200000000001637</v>
+        <v>70.40000000001601</v>
       </c>
     </row>
     <row r="12">
@@ -843,13 +905,13 @@
         <v>1.75</v>
       </c>
       <c r="B12" t="n">
-        <v>0.1000000000000227</v>
+        <v>0.2000000000000455</v>
       </c>
       <c r="C12" t="n">
-        <v>1.75</v>
+        <v>2.25</v>
       </c>
       <c r="D12" t="n">
-        <v>5.000000000001137</v>
+        <v>4.700000000001069</v>
       </c>
     </row>
     <row r="13">
@@ -860,10 +922,10 @@
         <v>0.3000000000000682</v>
       </c>
       <c r="C13" t="n">
-        <v>-1.75</v>
+        <v>-2.25</v>
       </c>
       <c r="D13" t="n">
-        <v>5.800000000001319</v>
+        <v>4.400000000001</v>
       </c>
     </row>
     <row r="14">
@@ -871,13 +933,13 @@
         <v>2</v>
       </c>
       <c r="B14" t="n">
-        <v>0.1000000000000227</v>
+        <v>0.2000000000000455</v>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="D14" t="n">
-        <v>4.600000000001046</v>
+        <v>28.50000000000648</v>
       </c>
     </row>
     <row r="15">
@@ -885,13 +947,13 @@
         <v>-2</v>
       </c>
       <c r="B15" t="n">
-        <v>0.3000000000000682</v>
+        <v>0.2000000000000455</v>
       </c>
       <c r="C15" t="n">
-        <v>-2</v>
+        <v>-2.5</v>
       </c>
       <c r="D15" t="n">
-        <v>5.700000000001296</v>
+        <v>4.100000000000932</v>
       </c>
     </row>
     <row r="16">
@@ -899,13 +961,69 @@
         <v>2.25</v>
       </c>
       <c r="B16" t="n">
-        <v>0.1000000000000227</v>
+        <v>0.3000000000000682</v>
       </c>
       <c r="C16" t="n">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="D16" t="n">
-        <v>4.700000000001069</v>
+        <v>4.799999999995634</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>-2.25</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0.4000000000000909</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.4000000000000909</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B20" t="n">
+        <v>0.3000000000000682</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="B21" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" t="n">
+        <v>0.3999999999996362</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>-3</v>
+      </c>
+      <c r="B23" t="n">
+        <v>0.1999999999998181</v>
       </c>
     </row>
   </sheetData>
@@ -919,6 +1037,730 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Accel_Value</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Response_Time</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Accel_Value</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Accel/Decel_Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.1000000000000014</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>296.5000000000104</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.2999999999999829</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="D3" t="n">
+        <v>140.3000000000319</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.1000000000000227</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>9.200000000002092</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.3000000000000682</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>8.500000000001933</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0.4000000000000909</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>60.80000000001382</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.3000000000000682</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>6.700000000001523</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.3000000000000682</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>4.800000000001091</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>-1</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.3000000000000682</v>
+      </c>
+      <c r="C9" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>5.10000000000116</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>5.000000000001137</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C11" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4.000000000000909</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" t="n">
+        <v>4.900000000001114</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>-2</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C13" t="n">
+        <v>-3</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3.400000000000773</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.3000000000000682</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.3000000000000682</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>-3</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.3000000000000682</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Accel_Value</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Response_Time</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Accel_Value</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Accel/Decel_Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.2000000000000028</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>89.49999999999704</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.3999999999999773</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="D3" t="n">
+        <v>37.59999999999786</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.2999999999999829</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>16.99999999999903</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.2999999999999829</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>19.50000000000401</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>9.100000000002069</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8.500000000001933</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.3000000000000682</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>6.300000000001432</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.3000000000000682</v>
+      </c>
+      <c r="C9" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>7.000000000001592</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>22.80000000000518</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>-2</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C11" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4.500000000001023</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D12" t="n">
+        <v>4.900000000001114</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C13" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="D13" t="n">
+        <v>4.200000000000955</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.3000000000000682</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" t="n">
+        <v>5.000000000001137</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>-3</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C15" t="n">
+        <v>-3</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3.600000000000819</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Accel_Value</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Response_Time</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Accel_Value</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Accel/Decel_Time</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.1000000000000014</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>87.99999999999551</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.3999999999999773</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-0.25</v>
+      </c>
+      <c r="D3" t="n">
+        <v>37.39999999999787</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.3999999999999773</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D4" t="n">
+        <v>17.19999999999902</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.3000000000000682</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>19.20000000000437</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>9.000000000002046</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>9.000000000002046</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.3000000000000682</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D8" t="n">
+        <v>6.400000000001455</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C9" t="n">
+        <v>-1.5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>8.40000000000191</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.3000000000000682</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="D10" t="n">
+        <v>5.300000000001205</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.3000000000000682</v>
+      </c>
+      <c r="C11" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="D11" t="n">
+        <v>5.500000000001251</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="n">
+        <v>4.700000000001069</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>-2</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C13" t="n">
+        <v>-2</v>
+      </c>
+      <c r="D13" t="n">
+        <v>4.900000000001114</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.3000000000000682</v>
+      </c>
+      <c r="C14" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D14" t="n">
+        <v>4.800000000001091</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C15" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="D15" t="n">
+        <v>4.200000000000955</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" t="n">
+        <v>4.900000000001114</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>-3</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.2000000000000455</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -949,13 +1791,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.1000000000000014</v>
+        <v>0.2000000000000028</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>111.2999999999966</v>
+        <v>89.49999999999704</v>
       </c>
     </row>
     <row r="3">
@@ -969,7 +1811,7 @@
         <v>-0.25</v>
       </c>
       <c r="D3" t="n">
-        <v>37.69999999999786</v>
+        <v>37.59999999999786</v>
       </c>
     </row>
     <row r="4">
@@ -983,7 +1825,7 @@
         <v>0.5</v>
       </c>
       <c r="D4" t="n">
-        <v>17.29999999999902</v>
+        <v>16.99999999999903</v>
       </c>
     </row>
     <row r="5">
@@ -991,13 +1833,13 @@
         <v>-0.5</v>
       </c>
       <c r="B5" t="n">
-        <v>0.3000000000000682</v>
+        <v>0.2999999999999829</v>
       </c>
       <c r="C5" t="n">
         <v>-0.5</v>
       </c>
       <c r="D5" t="n">
-        <v>24.80000000000564</v>
+        <v>19.50000000000401</v>
       </c>
     </row>
     <row r="6">
@@ -1005,13 +1847,13 @@
         <v>1</v>
       </c>
       <c r="B6" t="n">
-        <v>0.3000000000000682</v>
+        <v>0.2000000000000455</v>
       </c>
       <c r="C6" t="n">
         <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>9.000000000002046</v>
+        <v>9.100000000002069</v>
       </c>
     </row>
     <row r="7">
@@ -1025,7 +1867,7 @@
         <v>-1</v>
       </c>
       <c r="D7" t="n">
-        <v>8.700000000001978</v>
+        <v>8.500000000001933</v>
       </c>
     </row>
     <row r="8">
@@ -1039,7 +1881,7 @@
         <v>1.5</v>
       </c>
       <c r="D8" t="n">
-        <v>6.20000000000141</v>
+        <v>6.300000000001432</v>
       </c>
     </row>
     <row r="9">
@@ -1047,13 +1889,13 @@
         <v>-1.5</v>
       </c>
       <c r="B9" t="n">
-        <v>0.2000000000000455</v>
+        <v>0.3000000000000682</v>
       </c>
       <c r="C9" t="n">
         <v>-1.5</v>
       </c>
       <c r="D9" t="n">
-        <v>15.4000000000035</v>
+        <v>7.000000000001592</v>
       </c>
     </row>
     <row r="10">
@@ -1061,13 +1903,13 @@
         <v>2</v>
       </c>
       <c r="B10" t="n">
-        <v>0.3000000000000682</v>
+        <v>0.2000000000000455</v>
       </c>
       <c r="C10" t="n">
         <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>4.600000000001046</v>
+        <v>22.80000000000518</v>
       </c>
     </row>
     <row r="11">
@@ -1081,7 +1923,7 @@
         <v>-2</v>
       </c>
       <c r="D11" t="n">
-        <v>80.80000000001831</v>
+        <v>4.500000000001023</v>
       </c>
     </row>
     <row r="12">
@@ -1089,10 +1931,10 @@
         <v>2.5</v>
       </c>
       <c r="B12" t="n">
-        <v>0.4000000000000909</v>
+        <v>0.2000000000000455</v>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="D12" t="n">
         <v>4.900000000001114</v>
@@ -1106,10 +1948,10 @@
         <v>0.2000000000000455</v>
       </c>
       <c r="C13" t="n">
-        <v>-3</v>
+        <v>-2.5</v>
       </c>
       <c r="D13" t="n">
-        <v>3.30000000000075</v>
+        <v>4.200000000000955</v>
       </c>
     </row>
     <row r="14">
@@ -1117,10 +1959,14 @@
         <v>3</v>
       </c>
       <c r="B14" t="n">
-        <v>0.2000000000000455</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
+        <v>0.3000000000000682</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" t="n">
+        <v>5.000000000001137</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1129,8 +1975,12 @@
       <c r="B15" t="n">
         <v>0.2000000000000455</v>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
+      <c r="C15" t="n">
+        <v>-3</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3.600000000000819</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>